<commit_message>
changes for interests transactions and small fixes
</commit_message>
<xml_diff>
--- a/uploaded_files/Expenses.xlsx
+++ b/uploaded_files/Expenses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\REPORT\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\wealth_tracker_backend\uploaded_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667243F5-3156-4504-AA0A-5C3E39CACD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285BBD40-B1E0-40D2-B63D-C13B84D77FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{5EE44423-99DE-4A51-970D-BCA19FE5DD68}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{5EE44423-99DE-4A51-970D-BCA19FE5DD68}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="41">
   <si>
     <t>Date</t>
   </si>
@@ -123,6 +123,42 @@
   </si>
   <si>
     <t>Shoping</t>
+  </si>
+  <si>
+    <t>Kabini</t>
+  </si>
+  <si>
+    <t>Bali</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Coorg</t>
+  </si>
+  <si>
+    <t>Chikmagalur</t>
+  </si>
+  <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>Grocery</t>
+  </si>
+  <si>
+    <t>Dineout</t>
+  </si>
+  <si>
+    <t>Househelp</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Swimming</t>
   </si>
 </sst>
 </file>
@@ -478,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7B5B79-6329-4532-9353-B3B685E77AED}">
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -1849,6 +1885,336 @@
         <v>898</v>
       </c>
     </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B125" t="s">
+        <v>5</v>
+      </c>
+      <c r="C125">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B126" t="s">
+        <v>3</v>
+      </c>
+      <c r="C126">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B127" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B128" t="s">
+        <v>5</v>
+      </c>
+      <c r="C128">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B129" t="s">
+        <v>3</v>
+      </c>
+      <c r="C129">
+        <v>12774</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A130" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B130" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B131" t="s">
+        <v>5</v>
+      </c>
+      <c r="C131">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B132" t="s">
+        <v>3</v>
+      </c>
+      <c r="C132">
+        <v>15382</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B133" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B134" t="s">
+        <v>5</v>
+      </c>
+      <c r="C134">
+        <v>2587</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B135" t="s">
+        <v>3</v>
+      </c>
+      <c r="C135">
+        <v>12394</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A136" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B136" t="s">
+        <v>4</v>
+      </c>
+      <c r="C136">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A137" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B137" t="s">
+        <v>5</v>
+      </c>
+      <c r="C137">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A138" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B138" t="s">
+        <v>3</v>
+      </c>
+      <c r="C138">
+        <v>14480</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A139" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B139" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A140" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B140" t="s">
+        <v>5</v>
+      </c>
+      <c r="C140">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A141" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B141" t="s">
+        <v>3</v>
+      </c>
+      <c r="C141">
+        <v>12480</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A142" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B142" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A143" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B143" t="s">
+        <v>5</v>
+      </c>
+      <c r="C143">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A144" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B144" t="s">
+        <v>3</v>
+      </c>
+      <c r="C144">
+        <v>14600</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A145" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B145" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A146" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B146" t="s">
+        <v>5</v>
+      </c>
+      <c r="C146">
+        <v>3076</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A147" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B147" t="s">
+        <v>3</v>
+      </c>
+      <c r="C147">
+        <v>13120</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A148" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B148" t="s">
+        <v>4</v>
+      </c>
+      <c r="C148">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A149" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B149" t="s">
+        <v>5</v>
+      </c>
+      <c r="C149">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A150" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B150" t="s">
+        <v>3</v>
+      </c>
+      <c r="C150">
+        <v>14340</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A151" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B151" t="s">
+        <v>4</v>
+      </c>
+      <c r="C151">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A152" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B152" t="s">
+        <v>5</v>
+      </c>
+      <c r="C152">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A153" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B153" t="s">
+        <v>3</v>
+      </c>
+      <c r="C153">
+        <v>17920</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A154" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B154" t="s">
+        <v>4</v>
+      </c>
+      <c r="C154">
+        <v>898</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1856,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD5ACB8-3AB7-4C72-B176-3DD6F1ABB43C}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -2016,6 +2382,61 @@
         <v>120222</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
+        <v>45849</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>45880</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16">
+        <v>13970</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
+        <v>45947</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17">
+        <v>116148</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
+        <v>45955</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18">
+        <v>14791</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
+        <v>45974</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19">
+        <v>7092</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2024,7 +2445,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF4B8399-0565-4B1A-80CE-05B6EB82813A}">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" style="1" bestFit="1" customWidth="1"/>
@@ -2646,6 +3067,732 @@
         <v>9321</v>
       </c>
     </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B57" t="s">
+        <v>34</v>
+      </c>
+      <c r="C57">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B58" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58">
+        <v>6200</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B59" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59">
+        <v>4346</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B60" t="s">
+        <v>36</v>
+      </c>
+      <c r="C60">
+        <v>4437</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B61" t="s">
+        <v>37</v>
+      </c>
+      <c r="C61">
+        <v>3861</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B62" t="s">
+        <v>38</v>
+      </c>
+      <c r="C62">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B63" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B65" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65">
+        <v>7281</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B66" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66">
+        <v>5300</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B67" t="s">
+        <v>37</v>
+      </c>
+      <c r="C67">
+        <v>5168</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B68" t="s">
+        <v>38</v>
+      </c>
+      <c r="C68">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69">
+        <v>5050</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B70" t="s">
+        <v>40</v>
+      </c>
+      <c r="C70">
+        <v>18676</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B71" t="s">
+        <v>34</v>
+      </c>
+      <c r="C71">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B72" t="s">
+        <v>10</v>
+      </c>
+      <c r="C72">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B73" t="s">
+        <v>35</v>
+      </c>
+      <c r="C73">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B74" t="s">
+        <v>36</v>
+      </c>
+      <c r="C74">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B75" t="s">
+        <v>37</v>
+      </c>
+      <c r="C75">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B76" t="s">
+        <v>38</v>
+      </c>
+      <c r="C76">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B77" t="s">
+        <v>34</v>
+      </c>
+      <c r="C77">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B78" t="s">
+        <v>10</v>
+      </c>
+      <c r="C78">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B79" t="s">
+        <v>35</v>
+      </c>
+      <c r="C79">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B80" t="s">
+        <v>36</v>
+      </c>
+      <c r="C80">
+        <v>3520</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B81" t="s">
+        <v>37</v>
+      </c>
+      <c r="C81">
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B82" t="s">
+        <v>38</v>
+      </c>
+      <c r="C82">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B83" t="s">
+        <v>9</v>
+      </c>
+      <c r="C83">
+        <v>7577</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B84" t="s">
+        <v>28</v>
+      </c>
+      <c r="C84">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B85" t="s">
+        <v>34</v>
+      </c>
+      <c r="C85">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B86" t="s">
+        <v>35</v>
+      </c>
+      <c r="C86">
+        <v>6700</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B87" t="s">
+        <v>36</v>
+      </c>
+      <c r="C87">
+        <v>3660</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B88" t="s">
+        <v>37</v>
+      </c>
+      <c r="C88">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B89" t="s">
+        <v>38</v>
+      </c>
+      <c r="C89">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B90" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B91" t="s">
+        <v>10</v>
+      </c>
+      <c r="C91">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B92" t="s">
+        <v>35</v>
+      </c>
+      <c r="C92">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B93" t="s">
+        <v>36</v>
+      </c>
+      <c r="C93">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B94" t="s">
+        <v>37</v>
+      </c>
+      <c r="C94">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B95" t="s">
+        <v>38</v>
+      </c>
+      <c r="C95">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B96" t="s">
+        <v>28</v>
+      </c>
+      <c r="C96">
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B97" t="s">
+        <v>34</v>
+      </c>
+      <c r="C97">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B98" t="s">
+        <v>35</v>
+      </c>
+      <c r="C98">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B99" t="s">
+        <v>36</v>
+      </c>
+      <c r="C99">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B100" t="s">
+        <v>37</v>
+      </c>
+      <c r="C100">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B101" t="s">
+        <v>38</v>
+      </c>
+      <c r="C101">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B102" t="s">
+        <v>34</v>
+      </c>
+      <c r="C102">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B103" t="s">
+        <v>10</v>
+      </c>
+      <c r="C103">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B104" t="s">
+        <v>35</v>
+      </c>
+      <c r="C104">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B105" t="s">
+        <v>36</v>
+      </c>
+      <c r="C105">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B106" t="s">
+        <v>37</v>
+      </c>
+      <c r="C106">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B107" t="s">
+        <v>38</v>
+      </c>
+      <c r="C107">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B108" t="s">
+        <v>28</v>
+      </c>
+      <c r="C108">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B109" t="s">
+        <v>9</v>
+      </c>
+      <c r="C109">
+        <v>13830</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B110" t="s">
+        <v>34</v>
+      </c>
+      <c r="C110">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B111" t="s">
+        <v>10</v>
+      </c>
+      <c r="C111">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B112" t="s">
+        <v>35</v>
+      </c>
+      <c r="C112">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B113" t="s">
+        <v>36</v>
+      </c>
+      <c r="C113">
+        <v>4100</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B114" t="s">
+        <v>37</v>
+      </c>
+      <c r="C114">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B115" t="s">
+        <v>38</v>
+      </c>
+      <c r="C115">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B116" t="s">
+        <v>11</v>
+      </c>
+      <c r="C116">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B117" t="s">
+        <v>34</v>
+      </c>
+      <c r="C117">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B118" t="s">
+        <v>10</v>
+      </c>
+      <c r="C118">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B119" t="s">
+        <v>35</v>
+      </c>
+      <c r="C119">
+        <v>7745</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B120" t="s">
+        <v>36</v>
+      </c>
+      <c r="C120">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B121" t="s">
+        <v>37</v>
+      </c>
+      <c r="C121">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B122" t="s">
+        <v>38</v>
+      </c>
+      <c r="C122">
+        <v>1500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>